<commit_message>
Match front and rear upper ties
</commit_message>
<xml_diff>
--- a/balcony-planter-riser/deliverables/bom/planter-riser-bom.xlsx
+++ b/balcony-planter-riser/deliverables/bom/planter-riser-bom.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BOM" sheetId="1" r:id="R3b354fd6f31242d2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="2" r:id="R1fc0b360500d4272"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Catalogue mapping" sheetId="3" r:id="Raf491b2c2e2446ca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cut plan" sheetId="4" r:id="Re2ef58cbfa354587"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BOM" sheetId="1" r:id="Rcace386b09a84fb3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="2" r:id="Rbbf969fa5ef9478a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Catalogue mapping" sheetId="3" r:id="R63fbac44ebb64336"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cut plan" sheetId="4" r:id="R6e13d5ac738440e9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -213,7 +213,7 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:personList xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:person displayName="User" id="{71D31858-2A00-47E8-9782-D98308E40E1D}"/>
+  <xltc:person displayName="User" id="{3519BA9F-506A-4291-8178-E1B3E860FD06}"/>
 </xltc:personList>
 </file>
 
@@ -238,7 +238,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="CatalogueMap" displayName="CatalogueMap" ref="A4:I15" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="CatalogueMap" displayName="CatalogueMap" ref="A4:I14" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="BOM codes"/>
     <x:tableColumn id="2" name="Retailer"/>
@@ -499,7 +499,7 @@
     </x:row>
     <x:row r="2" ht="25" customHeight="1">
       <x:c r="A2" s="5" t="str">
-        <x:v>Model v4 enclosure study - three main-frame sections: 90 x 45, 70 x 35 and 45 x 35</x:v>
+        <x:v>Model v5 enclosure study - matched 70 x 35 upper ties; direct-bearing uprights; 45 x 35 lower frame</x:v>
       </x:c>
       <x:c r="B2" s="5"/>
       <x:c r="C2" s="5"/>
@@ -553,7 +553,7 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="25" t="str">
-        <x:v>Top frame</x:v>
+        <x:v>Upper tie</x:v>
       </x:c>
       <x:c r="B5" s="25" t="str">
         <x:v>Main frame</x:v>
@@ -562,32 +562,32 @@
         <x:v>TB-01</x:v>
       </x:c>
       <x:c r="D5" s="25" t="str">
-        <x:v>Front load-bearing top bearer</x:v>
+        <x:v>Front upper tie aligned with joists (non-bearing)</x:v>
       </x:c>
       <x:c r="E5" s="25" t="str">
-        <x:v>H3 structural pine 90x45</x:v>
+        <x:v>H3 structural pine 70x35</x:v>
       </x:c>
       <x:c r="F5" s="26" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G5" s="26" t="n">
-        <x:v>900</x:v>
+        <x:v>760</x:v>
       </x:c>
       <x:c r="H5" s="26" t="n">
-        <x:v>90</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="I5" s="26" t="n">
-        <x:v>45</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="J5" s="27" t="n">
         <x:f>IF(OR(F5="",G5=""),"",F5*G5/1000)</x:f>
-        <x:v>0.9</x:v>
+        <x:v>0.76</x:v>
       </x:c>
       <x:c r="K5" s="25" t="str">
         <x:v>Provisional</x:v>
       </x:c>
       <x:c r="L5" s="25" t="str">
-        <x:v>Carries the two front planter feet</x:v>
+        <x:v>Matches TB-02 between the full-height front uprights</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -649,7 +649,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G7" s="29" t="n">
-        <x:v>370</x:v>
+        <x:v>380</x:v>
       </x:c>
       <x:c r="H7" s="29" t="n">
         <x:v>70</x:v>
@@ -659,13 +659,13 @@
       </x:c>
       <x:c r="J7" s="30" t="n">
         <x:f>IF(OR(F7="",G7=""),"",F7*G7/1000)</x:f>
-        <x:v>1.11</x:v>
+        <x:v>1.14</x:v>
       </x:c>
       <x:c r="K7" s="28" t="str">
         <x:v>Provisional</x:v>
       </x:c>
       <x:c r="L7" s="28" t="str">
-        <x:v>Close the front-bearer-to-rear-tie span without a gap</x:v>
+        <x:v>Span cleanly between the matched 35 mm-thick upper ties</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -688,7 +688,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G8" s="29" t="n">
-        <x:v>534</x:v>
+        <x:v>514</x:v>
       </x:c>
       <x:c r="H8" s="29" t="n">
         <x:v>70</x:v>
@@ -698,7 +698,7 @@
       </x:c>
       <x:c r="J8" s="30" t="n">
         <x:f>IF(OR(F8="",G8=""),"",F8*G8/1000)</x:f>
-        <x:v>2.136</x:v>
+        <x:v>2.056</x:v>
       </x:c>
       <x:c r="K8" s="28" t="str">
         <x:v>Provisional</x:v>
@@ -1363,7 +1363,7 @@
         <x:v>Detail required</x:v>
       </x:c>
       <x:c r="L25" s="28" t="str">
-        <x:v>One flush strap bridges each planter post, top bearer and riser upright</x:v>
+        <x:v>One flush strap joins each planter post to its corresponding full-height upright; the upper tie remains non-bearing</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
@@ -1495,7 +1495,7 @@
       <x:c r="I29" s="21"/>
       <x:c r="J29" s="21" t="n">
         <x:f>SUM(J5:J28)</x:f>
-        <x:v>17.512000000000004</x:v>
+        <x:v>17.322000000000003</x:v>
       </x:c>
       <x:c r="K29" s="17" t="str">
         <x:v>Not a purchase quantity</x:v>
@@ -1511,7 +1511,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R230039fdb3794928"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R34ce2097676749fc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1550,7 +1550,7 @@
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="25" t="str">
-        <x:v>Clear space below top bearer</x:v>
+        <x:v>Clear space below upper ties</x:v>
       </x:c>
       <x:c r="B4" s="25" t="n">
         <x:v>450</x:v>
@@ -1559,26 +1559,26 @@
         <x:v>User confirmed</x:v>
       </x:c>
       <x:c r="D4" s="25" t="str">
-        <x:v>Sets leg length; top bearer adds 90 mm to planter lift</x:v>
+        <x:v>Sets upright length; the 70 mm tie depth brings the planter base to 520 mm above the balcony</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="28" t="str">
-        <x:v>Front top bearer section</x:v>
+        <x:v>Upper tie section</x:v>
       </x:c>
       <x:c r="B5" s="28" t="str">
-        <x:v>90 x 45 mm</x:v>
+        <x:v>70 x 35 mm</x:v>
       </x:c>
       <x:c r="C5" s="28" t="str">
-        <x:v>Provisional</x:v>
+        <x:v>Optimised</x:v>
       </x:c>
       <x:c r="D5" s="28" t="str">
-        <x:v>Retained for the 900 mm front load-carrying span</x:v>
+        <x:v>TB-01 and TB-02 match and remain outside the direct planter bearing path</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="28" t="str">
-        <x:v>Secondary frame section</x:v>
+        <x:v>Primary frame section</x:v>
       </x:c>
       <x:c r="B6" s="28" t="str">
         <x:v>70 x 35 mm</x:v>
@@ -1587,7 +1587,7 @@
         <x:v>Optimised</x:v>
       </x:c>
       <x:c r="D6" s="28" t="str">
-        <x:v>Full-height uprights, rear upper tie, short top joists and floor bearer</x:v>
+        <x:v>Full-height uprights, matched upper ties, short top joists and floor bearer</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -1749,13 +1749,13 @@
         <x:v>Stock families</x:v>
       </x:c>
       <x:c r="B18" s="31" t="str">
-        <x:v>90x45; 70x35; 45x35; 42x19; sheet material</x:v>
+        <x:v>70x35; 45x35; 42x19; sheet material</x:v>
       </x:c>
       <x:c r="C18" s="31" t="str">
         <x:v>Optimised</x:v>
       </x:c>
       <x:c r="D18" s="31" t="str">
-        <x:v>Large timber is restricted to the front load-bearing member</x:v>
+        <x:v>No 90 x 45 framing remains; both upper ties use the primary 70 x 35 stock</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1838,294 +1838,267 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="25" t="str">
-        <x:v>TB-01</x:v>
+        <x:v>TB, TJ, LG, FS</x:v>
       </x:c>
       <x:c r="B5" s="25" t="str">
         <x:v>Bowens</x:v>
       </x:c>
       <x:c r="C5" s="25" t="str">
-        <x:v>90x45 mm Treated Pine MGP10 H3 LOSP Kiln Dried</x:v>
+        <x:v>70x35 mm Treated Pine MGP10 H3 LOSP Kiln Dried</x:v>
       </x:c>
       <x:c r="D5" s="25" t="str">
-        <x:v>SKU MLPT090045</x:v>
+        <x:v>SKU MLPT070035</x:v>
       </x:c>
       <x:c r="E5" s="25" t="str">
         <x:v>2.4 m</x:v>
       </x:c>
       <x:c r="F5" s="27" t="n">
-        <x:v>1</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="G5" s="27"/>
       <x:c r="H5" s="25" t="str">
-        <x:v>https://www.bowens.com.au/p/90x45mm-pine-mgp10-h3-losp-kiln-dried/</x:v>
+        <x:v>https://www.bowens.com.au/p/70x35mm-pine-mgp10-h3-losp-kiln-dried/</x:v>
       </x:c>
       <x:c r="I5" s="25" t="str">
-        <x:v>Only the front load-bearing top bearer uses this size</x:v>
+        <x:v>Three lengths cover four uprights, both matched upper ties, three top joists and the floor bearer</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="28" t="str">
-        <x:v>TB-02, TJ, LG, FS</x:v>
+        <x:v>BL, BE</x:v>
       </x:c>
       <x:c r="B6" s="28" t="str">
-        <x:v>Bowens</x:v>
+        <x:v>Either</x:v>
       </x:c>
       <x:c r="C6" s="28" t="str">
-        <x:v>70x35 mm Treated Pine MGP10 H3 LOSP Kiln Dried</x:v>
+        <x:v>H3 structural pine approximately 45x35 mm</x:v>
       </x:c>
       <x:c r="D6" s="28" t="str">
-        <x:v>SKU MLPT070035</x:v>
+        <x:v>Confirm exact item</x:v>
       </x:c>
       <x:c r="E6" s="28" t="str">
         <x:v>2.4 m</x:v>
       </x:c>
       <x:c r="F6" s="30" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G6" s="30"/>
-      <x:c r="H6" s="28" t="str">
-        <x:v>https://www.bowens.com.au/p/70x35mm-pine-mgp10-h3-losp-kiln-dried/</x:v>
-      </x:c>
+      <x:c r="H6" s="28" t="str"/>
       <x:c r="I6" s="28" t="str">
-        <x:v>Two lengths cover the four uprights, rear upper tie, top joists and floor bearer</x:v>
+        <x:v>Reduced lower frame section; confirm graded treated stock before purchase</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="28" t="str">
-        <x:v>BL, BE</x:v>
+        <x:v>SP, WL, HP, FL</x:v>
       </x:c>
       <x:c r="B7" s="28" t="str">
-        <x:v>Either</x:v>
+        <x:v>Bowens</x:v>
       </x:c>
       <x:c r="C7" s="28" t="str">
-        <x:v>H3 structural pine approximately 45x35 mm</x:v>
+        <x:v>Pine Plywood F8 Structural Black 12 mm</x:v>
       </x:c>
       <x:c r="D7" s="28" t="str">
-        <x:v>Confirm exact item</x:v>
+        <x:v>SKU PHPB122412</x:v>
       </x:c>
       <x:c r="E7" s="28" t="str">
-        <x:v>2.4 m</x:v>
+        <x:v>2400x1200x12 mm sheet</x:v>
       </x:c>
       <x:c r="F7" s="30" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="G7" s="30"/>
-      <x:c r="H7" s="28" t="str"/>
+      <x:c r="G7" s="30" t="n">
+        <x:v>75.9</x:v>
+      </x:c>
+      <x:c r="H7" s="28" t="str">
+        <x:v>https://www.bowens.com.au/p/pine-plywood-f8-structural-black/?size=2400x1200x12mm&amp;uom=ST%7C1</x:v>
+      </x:c>
       <x:c r="I7" s="28" t="str">
-        <x:v>Reduced lower frame section; confirm graded treated stock before purchase</x:v>
+        <x:v>Rear and side structural walls, hatch and floor nest from one common sheet; seal every cut edge</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="28" t="str">
-        <x:v>SP, WL, HP, FL</x:v>
+        <x:v>HF</x:v>
       </x:c>
       <x:c r="B8" s="28" t="str">
-        <x:v>Bowens</x:v>
+        <x:v>Either</x:v>
       </x:c>
       <x:c r="C8" s="28" t="str">
-        <x:v>Pine Plywood F8 Structural Black 12 mm</x:v>
+        <x:v>Exterior dressed timber approximately 42x19 mm</x:v>
       </x:c>
       <x:c r="D8" s="28" t="str">
-        <x:v>SKU PHPB122412</x:v>
+        <x:v>Confirm exact item</x:v>
       </x:c>
       <x:c r="E8" s="28" t="str">
-        <x:v>2400x1200x12 mm sheet</x:v>
+        <x:v>2.4 m</x:v>
       </x:c>
       <x:c r="F8" s="30" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="G8" s="30" t="n">
-        <x:v>75.9</x:v>
-      </x:c>
-      <x:c r="H8" s="28" t="str">
-        <x:v>https://www.bowens.com.au/p/pine-plywood-f8-structural-black/?size=2400x1200x12mm&amp;uom=ST%7C1</x:v>
-      </x:c>
+      <x:c r="G8" s="30"/>
+      <x:c r="H8" s="28" t="str"/>
       <x:c r="I8" s="28" t="str">
-        <x:v>Rear and side structural walls, hatch and floor nest from one common sheet; seal every cut edge</x:v>
+        <x:v>Non-structural hatch stock; exact individual product still to be selected</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="28" t="str">
-        <x:v>HF</x:v>
+        <x:v>TJ connectors</x:v>
       </x:c>
       <x:c r="B9" s="28" t="str">
-        <x:v>Either</x:v>
+        <x:v>Bunnings</x:v>
       </x:c>
       <x:c r="C9" s="28" t="str">
-        <x:v>Exterior dressed timber approximately 42x19 mm</x:v>
+        <x:v>Rated connector to suit 35 x 70 mm joists</x:v>
       </x:c>
       <x:c r="D9" s="28" t="str">
         <x:v>Confirm exact item</x:v>
       </x:c>
       <x:c r="E9" s="28" t="str">
-        <x:v>2.4 m</x:v>
+        <x:v>Each</x:v>
       </x:c>
       <x:c r="F9" s="30" t="n">
-        <x:v>1</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="G9" s="30"/>
       <x:c r="H9" s="28" t="str"/>
       <x:c r="I9" s="28" t="str">
-        <x:v>Non-structural hatch stock; exact individual product still to be selected</x:v>
+        <x:v>Old 45 x 90 Pryda hanger does not fit the optimised joists</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="28" t="str">
-        <x:v>TJ connectors</x:v>
+        <x:v>Connector fasteners</x:v>
       </x:c>
       <x:c r="B10" s="28" t="str">
         <x:v>Bunnings</x:v>
       </x:c>
       <x:c r="C10" s="28" t="str">
-        <x:v>Rated connector to suit 35 x 70 mm joists</x:v>
+        <x:v>Pryda Timber Connector Screw 12G x 35 mm Hex Head</x:v>
       </x:c>
       <x:c r="D10" s="28" t="str">
-        <x:v>Confirm exact item</x:v>
+        <x:v>I/N 0084754</x:v>
       </x:c>
       <x:c r="E10" s="28" t="str">
-        <x:v>Each</x:v>
+        <x:v>Pack of 50</x:v>
       </x:c>
       <x:c r="F10" s="30" t="n">
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G10" s="30"/>
-      <x:c r="H10" s="28" t="str"/>
+      <x:c r="H10" s="28" t="str">
+        <x:v>https://www.bunnings.com.au/pryda-timber-connector-screw-12g-x-35mm-hex-head-pack-50_p0084754</x:v>
+      </x:c>
       <x:c r="I10" s="28" t="str">
-        <x:v>Old 45 x 90 Pryda hanger does not fit the optimised joists</x:v>
+        <x:v>Use only where permitted by the selected connector schedule</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="28" t="str">
-        <x:v>Connector fasteners</x:v>
+        <x:v>ST-01 - ST-04</x:v>
       </x:c>
       <x:c r="B11" s="28" t="str">
-        <x:v>Bunnings</x:v>
+        <x:v>Either</x:v>
       </x:c>
       <x:c r="C11" s="28" t="str">
-        <x:v>Pryda Timber Connector Screw 12G x 35 mm Hex Head</x:v>
+        <x:v>Galvanised flat splice strap approximately 300 x 40 x 3 mm</x:v>
       </x:c>
       <x:c r="D11" s="28" t="str">
-        <x:v>I/N 0084754</x:v>
+        <x:v>Confirm exact item</x:v>
       </x:c>
       <x:c r="E11" s="28" t="str">
-        <x:v>Pack of 50</x:v>
+        <x:v>Each</x:v>
       </x:c>
       <x:c r="F11" s="30" t="n">
-        <x:v>1</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="G11" s="30"/>
-      <x:c r="H11" s="28" t="str">
-        <x:v>https://www.bunnings.com.au/pryda-timber-connector-screw-12g-x-35mm-hex-head-pack-50_p0084754</x:v>
-      </x:c>
+      <x:c r="H11" s="28" t="str"/>
       <x:c r="I11" s="28" t="str">
-        <x:v>Use only where permitted by the selected connector schedule</x:v>
+        <x:v>Concealed detail replaces timber capture blocks and angle brackets; drill pattern must avoid timber edges</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="28" t="str">
-        <x:v>ST-01 - ST-04</x:v>
+        <x:v>ST fixing bolts</x:v>
       </x:c>
       <x:c r="B12" s="28" t="str">
-        <x:v>Either</x:v>
+        <x:v>Bunnings</x:v>
       </x:c>
       <x:c r="C12" s="28" t="str">
-        <x:v>Galvanised flat splice strap approximately 300 x 40 x 3 mm</x:v>
+        <x:v>Zenith M8 x 60 mm Hot Dipped Galvanised Cup Head Bolt and Nut</x:v>
       </x:c>
       <x:c r="D12" s="28" t="str">
-        <x:v>Confirm exact item</x:v>
+        <x:v>I/N 2310034</x:v>
       </x:c>
       <x:c r="E12" s="28" t="str">
         <x:v>Each</x:v>
       </x:c>
       <x:c r="F12" s="30" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="G12" s="30"/>
-      <x:c r="H12" s="28" t="str"/>
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="G12" s="30" t="n">
+        <x:v>0.74</x:v>
+      </x:c>
+      <x:c r="H12" s="28" t="str">
+        <x:v>https://www.bunnings.com.au/zenith-m8-x-60mm-hot-dipped-galvanised-cup-head-bolt-and-nut-each_p2310034</x:v>
+      </x:c>
       <x:c r="I12" s="28" t="str">
-        <x:v>Concealed detail replaces timber capture blocks and angle brackets; drill pattern must avoid timber edges</x:v>
+        <x:v>Two per strap plus suitable M8 galvanised washers; verify final grip length</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="28" t="str">
-        <x:v>ST fixing bolts</x:v>
+        <x:v>IP-01 - IP-04</x:v>
       </x:c>
       <x:c r="B13" s="28" t="str">
-        <x:v>Bunnings</x:v>
+        <x:v>Either</x:v>
       </x:c>
       <x:c r="C13" s="28" t="str">
-        <x:v>Zenith M8 x 60 mm Hot Dipped Galvanised Cup Head Bolt and Nut</x:v>
+        <x:v>Exterior EPDM isolation pad approximately 70 x 45 x 6 mm</x:v>
       </x:c>
       <x:c r="D13" s="28" t="str">
-        <x:v>I/N 2310034</x:v>
+        <x:v>Confirm exact item</x:v>
       </x:c>
       <x:c r="E13" s="28" t="str">
         <x:v>Each</x:v>
       </x:c>
       <x:c r="F13" s="30" t="n">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="G13" s="30" t="n">
-        <x:v>0.74</x:v>
-      </x:c>
-      <x:c r="H13" s="28" t="str">
-        <x:v>https://www.bunnings.com.au/zenith-m8-x-60mm-hot-dipped-galvanised-cup-head-bolt-and-nut-each_p2310034</x:v>
-      </x:c>
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="G13" s="30"/>
+      <x:c r="H13" s="28" t="str"/>
       <x:c r="I13" s="28" t="str">
-        <x:v>Two per strap plus suitable M8 galvanised washers; verify final grip length</x:v>
+        <x:v>Default option; can be cut from a suitable exterior rubber sheet</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
-      <x:c r="A14" s="28" t="str">
-        <x:v>IP-01 - IP-04</x:v>
-      </x:c>
-      <x:c r="B14" s="28" t="str">
-        <x:v>Either</x:v>
-      </x:c>
-      <x:c r="C14" s="28" t="str">
-        <x:v>Exterior EPDM isolation pad approximately 70 x 45 x 6 mm</x:v>
-      </x:c>
-      <x:c r="D14" s="28" t="str">
-        <x:v>Confirm exact item</x:v>
-      </x:c>
-      <x:c r="E14" s="28" t="str">
+      <x:c r="A14" s="31" t="str">
+        <x:v>PD-01 - PD-04</x:v>
+      </x:c>
+      <x:c r="B14" s="31" t="str">
+        <x:v>Bunnings</x:v>
+      </x:c>
+      <x:c r="C14" s="31" t="str">
+        <x:v>Builders Edge 25-40 mm Minifoot Pedestal Feet</x:v>
+      </x:c>
+      <x:c r="D14" s="31" t="str">
+        <x:v>I/N 2450073</x:v>
+      </x:c>
+      <x:c r="E14" s="31" t="str">
         <x:v>Each</x:v>
       </x:c>
-      <x:c r="F14" s="30" t="n">
+      <x:c r="F14" s="33" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="G14" s="30"/>
-      <x:c r="H14" s="28" t="str"/>
-      <x:c r="I14" s="28" t="str">
-        <x:v>Default option; can be cut from a suitable exterior rubber sheet</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15">
-      <x:c r="A15" s="31" t="str">
-        <x:v>PD-01 - PD-04</x:v>
-      </x:c>
-      <x:c r="B15" s="31" t="str">
-        <x:v>Bunnings</x:v>
-      </x:c>
-      <x:c r="C15" s="31" t="str">
-        <x:v>Builders Edge 25-40 mm Minifoot Pedestal Feet</x:v>
-      </x:c>
-      <x:c r="D15" s="31" t="str">
-        <x:v>I/N 2450073</x:v>
-      </x:c>
-      <x:c r="E15" s="31" t="str">
-        <x:v>Each</x:v>
-      </x:c>
-      <x:c r="F15" s="33" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="G15" s="33" t="n">
+      <x:c r="G14" s="33" t="n">
         <x:v>9.14</x:v>
       </x:c>
-      <x:c r="H15" s="31" t="str">
+      <x:c r="H14" s="31" t="str">
         <x:v>https://www.bunnings.com.au/builders-edge-25-40mm-minifoot-pedestal-feet_p2450073</x:v>
       </x:c>
-      <x:c r="I15" s="31" t="str">
+      <x:c r="I14" s="31" t="str">
         <x:v>Optional only if balcony fall requires levelling</x:v>
       </x:c>
     </x:row>
@@ -2136,7 +2109,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R441cc4632b9c418b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R75246911019446d0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2219,36 +2192,36 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="13" t="str">
-        <x:v>90-01</x:v>
+        <x:v>70-01</x:v>
       </x:c>
       <x:c r="B5" s="13" t="str">
-        <x:v>MLPT090045 - 90x45 H3 LOSP</x:v>
+        <x:v>MLPT070035 - 70x35 H3 LOSP</x:v>
       </x:c>
       <x:c r="C5" s="22" t="n">
         <x:v>2400</x:v>
       </x:c>
       <x:c r="D5" s="22" t="str">
-        <x:v>TB-01</x:v>
+        <x:v>LG-01</x:v>
       </x:c>
       <x:c r="E5" s="22" t="n">
-        <x:v>900</x:v>
+        <x:v>514</x:v>
       </x:c>
       <x:c r="F5" s="22" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G5" s="22" t="n">
-        <x:v>0</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="H5" s="22" t="n">
         <x:f>E5+G5</x:f>
-        <x:v>900</x:v>
+        <x:v>517</x:v>
       </x:c>
       <x:c r="I5" s="22" t="n">
         <x:f>C5-SUMIFS($H$5:$H$27,$A$5:$A$27,A5)</x:f>
-        <x:v>1500</x:v>
+        <x:v>335</x:v>
       </x:c>
       <x:c r="J5" s="13" t="str">
-        <x:v>1500 mm remainder</x:v>
+        <x:v>Full-height direct-bearing upright</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -2262,24 +2235,24 @@
         <x:v>2400</x:v>
       </x:c>
       <x:c r="D6" s="23" t="str">
-        <x:v>LG-01</x:v>
+        <x:v>LG-02</x:v>
       </x:c>
       <x:c r="E6" s="23" t="n">
-        <x:v>534</x:v>
+        <x:v>514</x:v>
       </x:c>
       <x:c r="F6" s="23" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="G6" s="23" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="H6" s="23" t="n">
         <x:f>E6+G6</x:f>
-        <x:v>537</x:v>
+        <x:v>517</x:v>
       </x:c>
       <x:c r="I6" s="23" t="n">
         <x:f>C6-SUMIFS($H$5:$H$27,$A$5:$A$27,A6)</x:f>
-        <x:v>255</x:v>
+        <x:v>335</x:v>
       </x:c>
       <x:c r="J6" s="14" t="str">
         <x:v>Full-height direct-bearing upright</x:v>
@@ -2296,24 +2269,24 @@
         <x:v>2400</x:v>
       </x:c>
       <x:c r="D7" s="23" t="str">
-        <x:v>LG-02</x:v>
+        <x:v>LG-03</x:v>
       </x:c>
       <x:c r="E7" s="23" t="n">
-        <x:v>534</x:v>
+        <x:v>514</x:v>
       </x:c>
       <x:c r="F7" s="23" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="G7" s="23" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="H7" s="23" t="n">
         <x:f>E7+G7</x:f>
-        <x:v>537</x:v>
+        <x:v>517</x:v>
       </x:c>
       <x:c r="I7" s="23" t="n">
         <x:f>C7-SUMIFS($H$5:$H$27,$A$5:$A$27,A7)</x:f>
-        <x:v>255</x:v>
+        <x:v>335</x:v>
       </x:c>
       <x:c r="J7" s="14" t="str">
         <x:v>Full-height direct-bearing upright</x:v>
@@ -2330,32 +2303,32 @@
         <x:v>2400</x:v>
       </x:c>
       <x:c r="D8" s="23" t="str">
-        <x:v>LG-03</x:v>
+        <x:v>LG-04</x:v>
       </x:c>
       <x:c r="E8" s="23" t="n">
-        <x:v>534</x:v>
+        <x:v>514</x:v>
       </x:c>
       <x:c r="F8" s="23" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="G8" s="23" t="n">
-        <x:v>3</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="H8" s="23" t="n">
         <x:f>E8+G8</x:f>
-        <x:v>537</x:v>
+        <x:v>514</x:v>
       </x:c>
       <x:c r="I8" s="23" t="n">
         <x:f>C8-SUMIFS($H$5:$H$27,$A$5:$A$27,A8)</x:f>
-        <x:v>255</x:v>
+        <x:v>335</x:v>
       </x:c>
       <x:c r="J8" s="14" t="str">
-        <x:v>Full-height direct-bearing upright</x:v>
+        <x:v>335 mm remainder</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="14" t="str">
-        <x:v>70-01</x:v>
+        <x:v>70-02</x:v>
       </x:c>
       <x:c r="B9" s="14" t="str">
         <x:v>MLPT070035 - 70x35 H3 LOSP</x:v>
@@ -2364,27 +2337,27 @@
         <x:v>2400</x:v>
       </x:c>
       <x:c r="D9" s="23" t="str">
-        <x:v>LG-04</x:v>
+        <x:v>TB-01</x:v>
       </x:c>
       <x:c r="E9" s="23" t="n">
-        <x:v>534</x:v>
+        <x:v>760</x:v>
       </x:c>
       <x:c r="F9" s="23" t="n">
-        <x:v>4</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G9" s="23" t="n">
-        <x:v>0</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="H9" s="23" t="n">
         <x:f>E9+G9</x:f>
-        <x:v>534</x:v>
+        <x:v>763</x:v>
       </x:c>
       <x:c r="I9" s="23" t="n">
         <x:f>C9-SUMIFS($H$5:$H$27,$A$5:$A$27,A9)</x:f>
-        <x:v>255</x:v>
+        <x:v>111</x:v>
       </x:c>
       <x:c r="J9" s="14" t="str">
-        <x:v>255 mm remainder</x:v>
+        <x:v>Non-bearing front tie aligned with joists</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -2404,7 +2377,7 @@
         <x:v>760</x:v>
       </x:c>
       <x:c r="F10" s="23" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="G10" s="23" t="n">
         <x:v>3</x:v>
@@ -2415,10 +2388,10 @@
       </x:c>
       <x:c r="I10" s="23" t="n">
         <x:f>C10-SUMIFS($H$5:$H$27,$A$5:$A$27,A10)</x:f>
-        <x:v>138</x:v>
+        <x:v>111</x:v>
       </x:c>
       <x:c r="J10" s="14" t="str">
-        <x:v>Non-bearing rear tie aligned with joists</x:v>
+        <x:v>Matching non-bearing rear tie</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -2435,21 +2408,21 @@
         <x:v>TJ-01</x:v>
       </x:c>
       <x:c r="E11" s="23" t="n">
-        <x:v>370</x:v>
+        <x:v>380</x:v>
       </x:c>
       <x:c r="F11" s="23" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="G11" s="23" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="H11" s="23" t="n">
         <x:f>E11+G11</x:f>
-        <x:v>373</x:v>
+        <x:v>383</x:v>
       </x:c>
       <x:c r="I11" s="23" t="n">
         <x:f>C11-SUMIFS($H$5:$H$27,$A$5:$A$27,A11)</x:f>
-        <x:v>138</x:v>
+        <x:v>111</x:v>
       </x:c>
       <x:c r="J11" s="14" t="str"/>
     </x:row>
@@ -2467,27 +2440,29 @@
         <x:v>TJ-02</x:v>
       </x:c>
       <x:c r="E12" s="23" t="n">
-        <x:v>370</x:v>
+        <x:v>380</x:v>
       </x:c>
       <x:c r="F12" s="23" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="G12" s="23" t="n">
-        <x:v>3</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="H12" s="23" t="n">
         <x:f>E12+G12</x:f>
-        <x:v>373</x:v>
+        <x:v>380</x:v>
       </x:c>
       <x:c r="I12" s="23" t="n">
         <x:f>C12-SUMIFS($H$5:$H$27,$A$5:$A$27,A12)</x:f>
-        <x:v>138</x:v>
-      </x:c>
-      <x:c r="J12" s="14" t="str"/>
+        <x:v>111</x:v>
+      </x:c>
+      <x:c r="J12" s="14" t="str">
+        <x:v>111 mm remainder</x:v>
+      </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="14" t="str">
-        <x:v>70-02</x:v>
+        <x:v>70-03</x:v>
       </x:c>
       <x:c r="B13" s="14" t="str">
         <x:v>MLPT070035 - 70x35 H3 LOSP</x:v>
@@ -2499,27 +2474,27 @@
         <x:v>TJ-03</x:v>
       </x:c>
       <x:c r="E13" s="23" t="n">
-        <x:v>370</x:v>
+        <x:v>380</x:v>
       </x:c>
       <x:c r="F13" s="23" t="n">
-        <x:v>4</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G13" s="23" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="H13" s="23" t="n">
         <x:f>E13+G13</x:f>
-        <x:v>373</x:v>
+        <x:v>383</x:v>
       </x:c>
       <x:c r="I13" s="23" t="n">
         <x:f>C13-SUMIFS($H$5:$H$27,$A$5:$A$27,A13)</x:f>
-        <x:v>138</x:v>
+        <x:v>1637</x:v>
       </x:c>
       <x:c r="J13" s="14" t="str"/>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="14" t="str">
-        <x:v>70-02</x:v>
+        <x:v>70-03</x:v>
       </x:c>
       <x:c r="B14" s="14" t="str">
         <x:v>MLPT070035 - 70x35 H3 LOSP</x:v>
@@ -2534,7 +2509,7 @@
         <x:v>380</x:v>
       </x:c>
       <x:c r="F14" s="23" t="n">
-        <x:v>5</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="G14" s="23" t="n">
         <x:v>0</x:v>
@@ -2545,10 +2520,10 @@
       </x:c>
       <x:c r="I14" s="23" t="n">
         <x:f>C14-SUMIFS($H$5:$H$27,$A$5:$A$27,A14)</x:f>
-        <x:v>138</x:v>
+        <x:v>1637</x:v>
       </x:c>
       <x:c r="J14" s="14" t="str">
-        <x:v>138 mm remainder</x:v>
+        <x:v>1637 mm remainder</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -2994,7 +2969,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R25aca44fdf154bf0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R787e570e98274659"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>